<commit_message>
Require the sales-rep columns
Sales Rep 1 and 2 are part of the report this app exists to print, so they
are required rather than optional. An export lacking them is the wrong
report and is now rejected by name instead of quietly producing a report
with two blank columns.

The test fixture gains both columns so it mirrors the report variant in
use rather than the export that happened to be mailed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0172hCH2R7iZwY7JYBZ62CMC
</commit_message>
<xml_diff>
--- a/tests/fixtures/salesforce_olympia_sample.xlsx
+++ b/tests/fixtures/salesforce_olympia_sample.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:M24"/>
+  <dimension ref="A2:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -517,6 +517,16 @@
           <t>Assigned Service Resource: Name</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Sales Rep 1 Name</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Sales Rep 2 Name</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -568,6 +578,16 @@
           <t>Leona Miles</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Leona Miles</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Nolen Moore</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="D13" t="inlineStr">
@@ -609,6 +629,16 @@
           <t>Jose Perez</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Jose Perez</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Jorge Sande</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="D14" t="inlineStr">
@@ -650,6 +680,16 @@
           <t>Dale Porter</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Dale Porter</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Ana Ruiz</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="C15" t="inlineStr">
@@ -660,6 +700,16 @@
       <c r="I15" t="n">
         <v>116491.82</v>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Erin Walsh</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Nolen Moore</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="C16" t="inlineStr">
@@ -667,6 +717,16 @@
           <t>Install Issue</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Leona Miles</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Nolen Moore</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="D17" t="inlineStr">
@@ -708,6 +768,16 @@
           <t>Leona Miles</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Jose Perez</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Jorge Sande</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="D18" t="inlineStr">
@@ -749,6 +819,16 @@
           <t>Jose Perez</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Dale Porter</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Ana Ruiz</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="C19" t="inlineStr">
@@ -759,6 +839,16 @@
       <c r="I19" t="n">
         <v>42950</v>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Erin Walsh</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Nolen Moore</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="C20" t="inlineStr">
@@ -766,6 +856,16 @@
           <t>On Hold</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Leona Miles</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Nolen Moore</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="D21" t="inlineStr">
@@ -807,6 +907,16 @@
           <t>Dale Porter</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Jose Perez</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Jorge Sande</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
@@ -858,6 +968,16 @@
           <t>Other Rep</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Dale Porter</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Ana Ruiz</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="D23" t="inlineStr">
@@ -899,6 +1019,16 @@
           <t>Other Rep</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Erin Walsh</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Nolen Moore</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
@@ -908,6 +1038,16 @@
       </c>
       <c r="I24" t="n">
         <v>379241.82</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Leona Miles</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Nolen Moore</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>